<commit_message>
Client BOM generated acc to #8
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/FLST_Digikey.xlsx
+++ b/Deliverables/BOM/FLST_Digikey.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24931"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\flst\Deliverables\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\flst\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5A847870-E048-49CA-B8C5-8B3578ADB5AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160"/>
   </bookViews>
   <sheets>
     <sheet name="Single Board" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -458,11 +457,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="165" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
@@ -770,15 +769,6 @@
     <xf numFmtId="165" fontId="7" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -794,9 +784,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -806,16 +793,28 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="170" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1098,7 +1097,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:R27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1121,24 +1120,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="33" t="s">
         <v>139</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="22"/>
-      <c r="M1" s="22"/>
-      <c r="N1" s="22"/>
-      <c r="O1" s="22"/>
-      <c r="P1" s="23"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
+      <c r="J1" s="34"/>
+      <c r="K1" s="34"/>
+      <c r="L1" s="34"/>
+      <c r="M1" s="34"/>
+      <c r="N1" s="34"/>
+      <c r="O1" s="34"/>
+      <c r="P1" s="35"/>
     </row>
     <row r="2" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -1194,34 +1193,34 @@
       <c r="A3" s="10">
         <v>1</v>
       </c>
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="27" t="s">
+      <c r="C3" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="D3" s="26" t="s">
+      <c r="D3" s="23" t="s">
         <v>65</v>
       </c>
-      <c r="E3" s="26" t="s">
+      <c r="E3" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="F3" s="26" t="s">
+      <c r="F3" s="23" t="s">
         <v>82</v>
       </c>
-      <c r="G3" s="26" t="s">
+      <c r="G3" s="23" t="s">
         <v>113</v>
       </c>
       <c r="H3" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="I3" s="26" t="s">
+      <c r="I3" s="23" t="s">
         <v>123</v>
       </c>
-      <c r="J3" s="24">
+      <c r="J3" s="21">
         <v>1</v>
       </c>
-      <c r="K3" s="24">
+      <c r="K3" s="21">
         <f>J3*5</f>
         <v>5</v>
       </c>
@@ -1247,32 +1246,32 @@
       <c r="A4" s="10">
         <v>2</v>
       </c>
-      <c r="B4" s="28"/>
-      <c r="C4" s="27" t="s">
+      <c r="B4" s="36"/>
+      <c r="C4" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="D4" s="26" t="s">
+      <c r="D4" s="23" t="s">
         <v>66</v>
       </c>
       <c r="E4" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="F4" s="26" t="s">
+      <c r="F4" s="23" t="s">
         <v>83</v>
       </c>
-      <c r="G4" s="26" t="s">
+      <c r="G4" s="23" t="s">
         <v>114</v>
       </c>
       <c r="H4" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="I4" s="26" t="s">
+      <c r="I4" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="J4" s="24">
+      <c r="J4" s="21">
         <v>1</v>
       </c>
-      <c r="K4" s="24">
+      <c r="K4" s="21">
         <f t="shared" ref="K4:K25" si="0">J4*5</f>
         <v>5</v>
       </c>
@@ -1280,7 +1279,7 @@
         <f t="shared" ref="L4:L25" si="1">K4*1.1*1</f>
         <v>5.5</v>
       </c>
-      <c r="M4" s="30" t="s">
+      <c r="M4" s="26" t="s">
         <v>42</v>
       </c>
       <c r="N4" s="5">
@@ -1298,32 +1297,32 @@
       <c r="A5" s="10">
         <v>3</v>
       </c>
-      <c r="B5" s="28"/>
-      <c r="C5" s="27" t="s">
+      <c r="B5" s="36"/>
+      <c r="C5" s="24" t="s">
         <v>45</v>
       </c>
-      <c r="D5" s="26" t="s">
+      <c r="D5" s="23" t="s">
         <v>67</v>
       </c>
-      <c r="E5" s="26" t="s">
+      <c r="E5" s="23" t="s">
         <v>84</v>
       </c>
-      <c r="F5" s="26" t="s">
+      <c r="F5" s="23" t="s">
         <v>85</v>
       </c>
-      <c r="G5" s="26" t="s">
+      <c r="G5" s="23" t="s">
         <v>9</v>
       </c>
       <c r="H5" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="I5" s="26" t="s">
+      <c r="I5" s="23" t="s">
         <v>124</v>
       </c>
-      <c r="J5" s="24">
+      <c r="J5" s="21">
         <v>1</v>
       </c>
-      <c r="K5" s="24">
+      <c r="K5" s="21">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
@@ -1349,32 +1348,32 @@
       <c r="A6" s="10">
         <v>4</v>
       </c>
-      <c r="B6" s="28"/>
-      <c r="C6" s="27" t="s">
+      <c r="B6" s="36"/>
+      <c r="C6" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="D6" s="26" t="s">
+      <c r="D6" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="E6" s="26" t="s">
+      <c r="E6" s="23" t="s">
         <v>84</v>
       </c>
-      <c r="F6" s="26" t="s">
+      <c r="F6" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="G6" s="26" t="s">
+      <c r="G6" s="23" t="s">
         <v>9</v>
       </c>
       <c r="H6" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="I6" s="26" t="s">
+      <c r="I6" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="J6" s="24">
+      <c r="J6" s="21">
         <v>2</v>
       </c>
-      <c r="K6" s="24">
+      <c r="K6" s="21">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
@@ -1400,32 +1399,32 @@
       <c r="A7" s="10">
         <v>5</v>
       </c>
-      <c r="B7" s="28"/>
-      <c r="C7" s="27" t="s">
+      <c r="B7" s="36"/>
+      <c r="C7" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="D7" s="26" t="s">
+      <c r="D7" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="E7" s="26" t="s">
+      <c r="E7" s="23" t="s">
         <v>84</v>
       </c>
-      <c r="F7" s="26" t="s">
+      <c r="F7" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="G7" s="26" t="s">
+      <c r="G7" s="23" t="s">
         <v>9</v>
       </c>
       <c r="H7" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="I7" s="26" t="s">
+      <c r="I7" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="J7" s="24">
+      <c r="J7" s="21">
         <v>1</v>
       </c>
-      <c r="K7" s="24">
+      <c r="K7" s="21">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
@@ -1451,34 +1450,34 @@
       <c r="A8" s="10">
         <v>6</v>
       </c>
-      <c r="B8" s="29" t="s">
+      <c r="B8" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="27" t="s">
+      <c r="C8" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="D8" s="26" t="s">
+      <c r="D8" s="23" t="s">
         <v>70</v>
       </c>
-      <c r="E8" s="26" t="s">
+      <c r="E8" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="F8" s="26" t="s">
+      <c r="F8" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="G8" s="26" t="s">
+      <c r="G8" s="23" t="s">
         <v>115</v>
       </c>
-      <c r="H8" s="31" t="s">
+      <c r="H8" s="27" t="s">
         <v>136</v>
       </c>
       <c r="I8" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="J8" s="24">
+      <c r="J8" s="21">
         <v>1</v>
       </c>
-      <c r="K8" s="24">
+      <c r="K8" s="21">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
@@ -1504,22 +1503,22 @@
       <c r="A9" s="10">
         <v>7</v>
       </c>
-      <c r="B9" s="28" t="s">
+      <c r="B9" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="C9" s="27" t="s">
+      <c r="C9" s="24" t="s">
         <v>49</v>
       </c>
-      <c r="D9" s="26" t="s">
+      <c r="D9" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="E9" s="26" t="s">
+      <c r="E9" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="F9" s="26" t="s">
+      <c r="F9" s="23" t="s">
         <v>90</v>
       </c>
-      <c r="G9" s="26" t="s">
+      <c r="G9" s="23" t="s">
         <v>116</v>
       </c>
       <c r="H9" s="8" t="s">
@@ -1528,10 +1527,10 @@
       <c r="I9" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="J9" s="24">
+      <c r="J9" s="21">
         <v>1</v>
       </c>
-      <c r="K9" s="24">
+      <c r="K9" s="21">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
@@ -1539,7 +1538,7 @@
         <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
-      <c r="M9" s="30" t="s">
+      <c r="M9" s="26" t="s">
         <v>137</v>
       </c>
       <c r="N9" s="5">
@@ -1557,20 +1556,20 @@
       <c r="A10" s="10">
         <v>8</v>
       </c>
-      <c r="B10" s="28"/>
-      <c r="C10" s="27" t="s">
+      <c r="B10" s="36"/>
+      <c r="C10" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="D10" s="26" t="s">
+      <c r="D10" s="23" t="s">
         <v>71</v>
       </c>
-      <c r="E10" s="26" t="s">
+      <c r="E10" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="F10" s="26">
+      <c r="F10" s="23">
         <v>61300211121</v>
       </c>
-      <c r="G10" s="26" t="s">
+      <c r="G10" s="23" t="s">
         <v>8</v>
       </c>
       <c r="H10" s="8" t="s">
@@ -1579,10 +1578,10 @@
       <c r="I10" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="J10" s="24">
+      <c r="J10" s="21">
         <v>10</v>
       </c>
-      <c r="K10" s="24">
+      <c r="K10" s="21">
         <f t="shared" si="0"/>
         <v>50</v>
       </c>
@@ -1608,34 +1607,34 @@
       <c r="A11" s="10">
         <v>9</v>
       </c>
-      <c r="B11" s="28" t="s">
+      <c r="B11" s="36" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="27" t="s">
+      <c r="C11" s="24" t="s">
         <v>50</v>
       </c>
-      <c r="D11" s="26" t="s">
+      <c r="D11" s="23" t="s">
         <v>32</v>
       </c>
       <c r="E11" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="F11" s="26" t="s">
+      <c r="F11" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="G11" s="26" t="s">
+      <c r="G11" s="23" t="s">
         <v>5</v>
       </c>
       <c r="H11" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="I11" s="26" t="s">
+      <c r="I11" s="23" t="s">
         <v>125</v>
       </c>
-      <c r="J11" s="24">
+      <c r="J11" s="21">
         <v>1</v>
       </c>
-      <c r="K11" s="24">
+      <c r="K11" s="21">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
@@ -1661,20 +1660,20 @@
       <c r="A12" s="10">
         <v>10</v>
       </c>
-      <c r="B12" s="28"/>
-      <c r="C12" s="27" t="s">
+      <c r="B12" s="36"/>
+      <c r="C12" s="24" t="s">
         <v>51</v>
       </c>
-      <c r="D12" s="26" t="s">
+      <c r="D12" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="E12" s="26" t="s">
+      <c r="E12" s="23" t="s">
         <v>92</v>
       </c>
-      <c r="F12" s="26" t="s">
+      <c r="F12" s="23" t="s">
         <v>93</v>
       </c>
-      <c r="G12" s="26" t="s">
+      <c r="G12" s="23" t="s">
         <v>5</v>
       </c>
       <c r="H12" s="8" t="s">
@@ -1683,10 +1682,10 @@
       <c r="I12" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="J12" s="24">
+      <c r="J12" s="21">
         <v>1</v>
       </c>
-      <c r="K12" s="24">
+      <c r="K12" s="21">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
@@ -1712,22 +1711,22 @@
       <c r="A13" s="10">
         <v>11</v>
       </c>
-      <c r="B13" s="29" t="s">
+      <c r="B13" s="25" t="s">
         <v>134</v>
       </c>
-      <c r="C13" s="27" t="s">
+      <c r="C13" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="D13" s="26" t="s">
+      <c r="D13" s="23" t="s">
         <v>72</v>
       </c>
-      <c r="E13" s="26" t="s">
+      <c r="E13" s="23" t="s">
         <v>95</v>
       </c>
-      <c r="F13" s="26" t="s">
+      <c r="F13" s="23" t="s">
         <v>96</v>
       </c>
-      <c r="G13" s="26" t="s">
+      <c r="G13" s="23" t="s">
         <v>6</v>
       </c>
       <c r="H13" s="8" t="s">
@@ -1736,10 +1735,10 @@
       <c r="I13" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="J13" s="24">
+      <c r="J13" s="21">
         <v>4</v>
       </c>
-      <c r="K13" s="24">
+      <c r="K13" s="21">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
@@ -1765,34 +1764,34 @@
       <c r="A14" s="10">
         <v>12</v>
       </c>
-      <c r="B14" s="28" t="s">
+      <c r="B14" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="C14" s="27" t="s">
+      <c r="C14" s="24" t="s">
         <v>53</v>
       </c>
-      <c r="D14" s="26" t="s">
+      <c r="D14" s="23" t="s">
         <v>73</v>
       </c>
-      <c r="E14" s="26" t="s">
+      <c r="E14" s="23" t="s">
         <v>97</v>
       </c>
-      <c r="F14" s="26" t="s">
+      <c r="F14" s="23" t="s">
         <v>98</v>
       </c>
-      <c r="G14" s="26" t="s">
+      <c r="G14" s="23" t="s">
         <v>117</v>
       </c>
       <c r="H14" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="I14" s="26" t="s">
+      <c r="I14" s="23" t="s">
         <v>126</v>
       </c>
-      <c r="J14" s="24">
+      <c r="J14" s="21">
         <v>1</v>
       </c>
-      <c r="K14" s="24">
+      <c r="K14" s="21">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
@@ -1800,7 +1799,7 @@
         <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
-      <c r="M14" s="30" t="s">
+      <c r="M14" s="26" t="s">
         <v>137</v>
       </c>
       <c r="N14" s="5">
@@ -1818,32 +1817,32 @@
       <c r="A15" s="10">
         <v>13</v>
       </c>
-      <c r="B15" s="28"/>
-      <c r="C15" s="27" t="s">
+      <c r="B15" s="36"/>
+      <c r="C15" s="24" t="s">
         <v>54</v>
       </c>
-      <c r="D15" s="26" t="s">
+      <c r="D15" s="23" t="s">
         <v>74</v>
       </c>
-      <c r="E15" s="26" t="s">
+      <c r="E15" s="23" t="s">
         <v>97</v>
       </c>
-      <c r="F15" s="26" t="s">
+      <c r="F15" s="23" t="s">
         <v>99</v>
       </c>
-      <c r="G15" s="26" t="s">
+      <c r="G15" s="23" t="s">
         <v>9</v>
       </c>
       <c r="H15" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="I15" s="26" t="s">
+      <c r="I15" s="23" t="s">
         <v>127</v>
       </c>
-      <c r="J15" s="24">
+      <c r="J15" s="21">
         <v>1</v>
       </c>
-      <c r="K15" s="24">
+      <c r="K15" s="21">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
@@ -1869,32 +1868,32 @@
       <c r="A16" s="10">
         <v>14</v>
       </c>
-      <c r="B16" s="28"/>
-      <c r="C16" s="27" t="s">
+      <c r="B16" s="36"/>
+      <c r="C16" s="24" t="s">
         <v>55</v>
       </c>
-      <c r="D16" s="26" t="s">
+      <c r="D16" s="23" t="s">
         <v>75</v>
       </c>
-      <c r="E16" s="26" t="s">
+      <c r="E16" s="23" t="s">
         <v>100</v>
       </c>
-      <c r="F16" s="26" t="s">
+      <c r="F16" s="23" t="s">
         <v>101</v>
       </c>
-      <c r="G16" s="26" t="s">
+      <c r="G16" s="23" t="s">
         <v>9</v>
       </c>
       <c r="H16" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="I16" s="26" t="s">
+      <c r="I16" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="J16" s="24">
+      <c r="J16" s="21">
         <v>4</v>
       </c>
-      <c r="K16" s="24">
+      <c r="K16" s="21">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
@@ -1920,32 +1919,32 @@
       <c r="A17" s="10">
         <v>15</v>
       </c>
-      <c r="B17" s="28"/>
-      <c r="C17" s="27" t="s">
+      <c r="B17" s="36"/>
+      <c r="C17" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="D17" s="26" t="s">
+      <c r="D17" s="23" t="s">
         <v>76</v>
       </c>
-      <c r="E17" s="26" t="s">
+      <c r="E17" s="23" t="s">
         <v>97</v>
       </c>
-      <c r="F17" s="26" t="s">
+      <c r="F17" s="23" t="s">
         <v>102</v>
       </c>
-      <c r="G17" s="26" t="s">
+      <c r="G17" s="23" t="s">
         <v>118</v>
       </c>
       <c r="H17" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="I17" s="26" t="s">
+      <c r="I17" s="23" t="s">
         <v>128</v>
       </c>
-      <c r="J17" s="24">
+      <c r="J17" s="21">
         <v>5</v>
       </c>
-      <c r="K17" s="24">
+      <c r="K17" s="21">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
@@ -1971,32 +1970,32 @@
       <c r="A18" s="10">
         <v>16</v>
       </c>
-      <c r="B18" s="28"/>
-      <c r="C18" s="27" t="s">
+      <c r="B18" s="36"/>
+      <c r="C18" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="D18" s="26" t="s">
+      <c r="D18" s="23" t="s">
         <v>77</v>
       </c>
-      <c r="E18" s="26" t="s">
+      <c r="E18" s="23" t="s">
         <v>97</v>
       </c>
-      <c r="F18" s="26" t="s">
+      <c r="F18" s="23" t="s">
         <v>103</v>
       </c>
-      <c r="G18" s="26" t="s">
+      <c r="G18" s="23" t="s">
         <v>9</v>
       </c>
       <c r="H18" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="I18" s="26" t="s">
+      <c r="I18" s="23" t="s">
         <v>129</v>
       </c>
-      <c r="J18" s="24">
+      <c r="J18" s="21">
         <v>5</v>
       </c>
-      <c r="K18" s="24">
+      <c r="K18" s="21">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
@@ -2022,32 +2021,32 @@
       <c r="A19" s="10">
         <v>17</v>
       </c>
-      <c r="B19" s="28"/>
-      <c r="C19" s="27" t="s">
+      <c r="B19" s="36"/>
+      <c r="C19" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="D19" s="26" t="s">
+      <c r="D19" s="23" t="s">
         <v>78</v>
       </c>
-      <c r="E19" s="26" t="s">
+      <c r="E19" s="23" t="s">
         <v>97</v>
       </c>
-      <c r="F19" s="26" t="s">
+      <c r="F19" s="23" t="s">
         <v>104</v>
       </c>
-      <c r="G19" s="26" t="s">
+      <c r="G19" s="23" t="s">
         <v>9</v>
       </c>
       <c r="H19" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="I19" s="26" t="s">
+      <c r="I19" s="23" t="s">
         <v>130</v>
       </c>
-      <c r="J19" s="24">
+      <c r="J19" s="21">
         <v>1</v>
       </c>
-      <c r="K19" s="24">
+      <c r="K19" s="21">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
@@ -2073,32 +2072,32 @@
       <c r="A20" s="10">
         <v>18</v>
       </c>
-      <c r="B20" s="28"/>
-      <c r="C20" s="27" t="s">
+      <c r="B20" s="36"/>
+      <c r="C20" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="D20" s="26" t="s">
+      <c r="D20" s="23" t="s">
         <v>79</v>
       </c>
-      <c r="E20" s="26" t="s">
+      <c r="E20" s="23" t="s">
         <v>97</v>
       </c>
-      <c r="F20" s="26" t="s">
+      <c r="F20" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="G20" s="26" t="s">
+      <c r="G20" s="23" t="s">
         <v>119</v>
       </c>
       <c r="H20" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="I20" s="26" t="s">
+      <c r="I20" s="23" t="s">
         <v>131</v>
       </c>
-      <c r="J20" s="24">
+      <c r="J20" s="21">
         <v>1</v>
       </c>
-      <c r="K20" s="24">
+      <c r="K20" s="21">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
@@ -2106,7 +2105,7 @@
         <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
-      <c r="M20" s="30" t="s">
+      <c r="M20" s="26" t="s">
         <v>138</v>
       </c>
       <c r="N20" s="12">
@@ -2124,22 +2123,22 @@
       <c r="A21" s="10">
         <v>19</v>
       </c>
-      <c r="B21" s="29" t="s">
+      <c r="B21" s="25" t="s">
         <v>135</v>
       </c>
-      <c r="C21" s="27" t="s">
+      <c r="C21" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="D21" s="26" t="s">
+      <c r="D21" s="23" t="s">
         <v>80</v>
       </c>
       <c r="E21" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="F21" s="26" t="s">
+      <c r="F21" s="23" t="s">
         <v>106</v>
       </c>
-      <c r="G21" s="26" t="s">
+      <c r="G21" s="23" t="s">
         <v>120</v>
       </c>
       <c r="H21" s="8" t="s">
@@ -2148,10 +2147,10 @@
       <c r="I21" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="J21" s="24">
+      <c r="J21" s="21">
         <v>1</v>
       </c>
-      <c r="K21" s="24">
+      <c r="K21" s="21">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
@@ -2159,7 +2158,7 @@
         <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
-      <c r="M21" s="30" t="s">
+      <c r="M21" s="26" t="s">
         <v>138</v>
       </c>
       <c r="N21" s="5">
@@ -2177,22 +2176,22 @@
       <c r="A22" s="10">
         <v>20</v>
       </c>
-      <c r="B22" s="28" t="s">
+      <c r="B22" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="C22" s="27" t="s">
+      <c r="C22" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="D22" s="26" t="s">
+      <c r="D22" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="E22" s="26" t="s">
+      <c r="E22" s="23" t="s">
         <v>107</v>
       </c>
-      <c r="F22" s="26" t="s">
+      <c r="F22" s="23" t="s">
         <v>108</v>
       </c>
-      <c r="G22" s="26" t="s">
+      <c r="G22" s="23" t="s">
         <v>36</v>
       </c>
       <c r="H22" s="8" t="s">
@@ -2201,10 +2200,10 @@
       <c r="I22" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="J22" s="24">
+      <c r="J22" s="21">
         <v>1</v>
       </c>
-      <c r="K22" s="24">
+      <c r="K22" s="21">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
@@ -2230,20 +2229,20 @@
       <c r="A23" s="10">
         <v>21</v>
       </c>
-      <c r="B23" s="28"/>
-      <c r="C23" s="27" t="s">
+      <c r="B23" s="36"/>
+      <c r="C23" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="D23" s="26" t="s">
+      <c r="D23" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="E23" s="26" t="s">
+      <c r="E23" s="23" t="s">
         <v>109</v>
       </c>
-      <c r="F23" s="26" t="s">
+      <c r="F23" s="23" t="s">
         <v>110</v>
       </c>
-      <c r="G23" s="26" t="s">
+      <c r="G23" s="23" t="s">
         <v>38</v>
       </c>
       <c r="H23" s="8" t="s">
@@ -2252,10 +2251,10 @@
       <c r="I23" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="J23" s="24">
+      <c r="J23" s="21">
         <v>1</v>
       </c>
-      <c r="K23" s="24">
+      <c r="K23" s="21">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
@@ -2281,20 +2280,20 @@
       <c r="A24" s="10">
         <v>22</v>
       </c>
-      <c r="B24" s="28"/>
-      <c r="C24" s="27" t="s">
+      <c r="B24" s="36"/>
+      <c r="C24" s="24" t="s">
         <v>63</v>
       </c>
-      <c r="D24" s="26" t="s">
+      <c r="D24" s="23" t="s">
         <v>39</v>
       </c>
       <c r="E24" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="F24" s="26" t="s">
+      <c r="F24" s="23" t="s">
         <v>111</v>
       </c>
-      <c r="G24" s="26" t="s">
+      <c r="G24" s="23" t="s">
         <v>121</v>
       </c>
       <c r="H24" s="8" t="s">
@@ -2303,10 +2302,10 @@
       <c r="I24" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="J24" s="24">
+      <c r="J24" s="21">
         <v>1</v>
       </c>
-      <c r="K24" s="24">
+      <c r="K24" s="21">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
@@ -2332,20 +2331,20 @@
       <c r="A25" s="10">
         <v>23</v>
       </c>
-      <c r="B25" s="28"/>
-      <c r="C25" s="27" t="s">
+      <c r="B25" s="36"/>
+      <c r="C25" s="24" t="s">
         <v>64</v>
       </c>
-      <c r="D25" s="26" t="s">
+      <c r="D25" s="23" t="s">
         <v>40</v>
       </c>
       <c r="E25" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="F25" s="26" t="s">
+      <c r="F25" s="23" t="s">
         <v>112</v>
       </c>
-      <c r="G25" s="26" t="s">
+      <c r="G25" s="23" t="s">
         <v>122</v>
       </c>
       <c r="H25" s="8" t="s">
@@ -2354,10 +2353,10 @@
       <c r="I25" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="J25" s="25">
+      <c r="J25" s="22">
         <v>1</v>
       </c>
-      <c r="K25" s="25">
+      <c r="K25" s="22">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
@@ -2365,7 +2364,7 @@
         <f t="shared" si="1"/>
         <v>5.5</v>
       </c>
-      <c r="M25" s="30" t="s">
+      <c r="M25" s="26" t="s">
         <v>138</v>
       </c>
       <c r="N25" s="5">
@@ -2380,26 +2379,26 @@
       <c r="R25" s="2"/>
     </row>
     <row r="26" spans="1:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="J26" s="33" t="s">
+      <c r="J26" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="K26" s="33"/>
-      <c r="L26" s="33"/>
-      <c r="M26" s="32"/>
-      <c r="N26" s="32"/>
-      <c r="O26" s="35">
+      <c r="K26" s="32"/>
+      <c r="L26" s="32"/>
+      <c r="M26" s="28"/>
+      <c r="N26" s="28"/>
+      <c r="O26" s="29">
         <f>SUM(O3:O25)</f>
         <v>96.008000000000024</v>
       </c>
     </row>
     <row r="27" spans="1:18" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="J27" s="34" t="s">
+      <c r="J27" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="K27" s="34"/>
-      <c r="L27" s="34"/>
+      <c r="K27" s="31"/>
+      <c r="L27" s="31"/>
       <c r="M27" s="13"/>
-      <c r="O27" s="36">
+      <c r="O27" s="30">
         <f>O26/5</f>
         <v>19.201600000000006</v>
       </c>
@@ -2506,23 +2505,23 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="M3" r:id="rId1" xr:uid="{0998FF86-454E-4391-A2E9-13C9F8F326B4}"/>
-    <hyperlink ref="M5" r:id="rId2" xr:uid="{3B6D6F3A-4401-45DF-91AC-8CD132CDC24F}"/>
-    <hyperlink ref="M6" r:id="rId3" xr:uid="{00062B14-3938-47E9-B80A-83919AE57DA0}"/>
-    <hyperlink ref="M7" r:id="rId4" xr:uid="{74F18444-7B44-44E9-A683-D5B5BF1697FA}"/>
-    <hyperlink ref="M8" r:id="rId5" xr:uid="{C78B20EF-4630-44B5-934D-EC4E3DD1DBD4}"/>
-    <hyperlink ref="M11" r:id="rId6" xr:uid="{DCB0E6C5-1DA5-4775-8C4E-F7FED8FB1385}"/>
-    <hyperlink ref="M12" r:id="rId7" xr:uid="{850E588C-928C-47B6-9A2E-C7890F83FDDF}"/>
-    <hyperlink ref="M13" r:id="rId8" xr:uid="{B62C7C90-7A79-4C8E-A7DE-C5153D4985A8}"/>
-    <hyperlink ref="M15" r:id="rId9" xr:uid="{72BDA2ED-6906-4257-AAE9-FD6081E7FDF2}"/>
-    <hyperlink ref="M16" r:id="rId10" xr:uid="{39EEF888-D759-4F6E-BBBD-7159327C8E3E}"/>
-    <hyperlink ref="M17" r:id="rId11" xr:uid="{283326BA-B823-4546-A209-FA092222FEBA}"/>
-    <hyperlink ref="M18" r:id="rId12" xr:uid="{4F5B6D8B-90C0-4300-939D-1FDC3AAFDDED}"/>
-    <hyperlink ref="M19" r:id="rId13" xr:uid="{582D0A97-B917-42FB-AE97-3094AA9D69B1}"/>
-    <hyperlink ref="M22" r:id="rId14" xr:uid="{9B83B3E9-C677-4B74-9ACD-A24AB630F44E}"/>
-    <hyperlink ref="M23" r:id="rId15" xr:uid="{9A11B207-9DC2-4177-9874-9ED848B488C6}"/>
-    <hyperlink ref="M24" r:id="rId16" xr:uid="{D905AE53-3B2F-49F2-9B2D-D8C32A6A5C6C}"/>
-    <hyperlink ref="M10" r:id="rId17" xr:uid="{D07B3FB0-0517-46C0-8D79-87AC7861CCB8}"/>
+    <hyperlink ref="M3" r:id="rId1"/>
+    <hyperlink ref="M5" r:id="rId2"/>
+    <hyperlink ref="M6" r:id="rId3"/>
+    <hyperlink ref="M7" r:id="rId4"/>
+    <hyperlink ref="M8" r:id="rId5"/>
+    <hyperlink ref="M11" r:id="rId6"/>
+    <hyperlink ref="M12" r:id="rId7"/>
+    <hyperlink ref="M13" r:id="rId8"/>
+    <hyperlink ref="M15" r:id="rId9"/>
+    <hyperlink ref="M16" r:id="rId10"/>
+    <hyperlink ref="M17" r:id="rId11"/>
+    <hyperlink ref="M18" r:id="rId12"/>
+    <hyperlink ref="M19" r:id="rId13"/>
+    <hyperlink ref="M22" r:id="rId14"/>
+    <hyperlink ref="M23" r:id="rId15"/>
+    <hyperlink ref="M24" r:id="rId16"/>
+    <hyperlink ref="M10" r:id="rId17"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId18"/>

</xml_diff>